<commit_message>
Refactor whatsapp_sender.spec to exclude binaries in EXE and add COLLECT for proper packaging; add failed_numbers.xlsx for tracking; include chromedriver-win64.zip and python311.dll for dependencies.
</commit_message>
<xml_diff>
--- a/WhatsAppSender/contacts.xlsx
+++ b/WhatsAppSender/contacts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yaser\OneDrive\Documents\PythonProjects\WhatsAppSendMessage\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\Python\WhatsAppSender\WhatsAppSender\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AAAAE4-8905-4E83-A221-4BF85E422F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72AB2C7C-A34C-4476-B6D2-C7DA6E0E4A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{9B310414-02F9-4358-91FC-CD1C7F3C01C7}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B310414-02F9-4358-91FC-CD1C7F3C01C7}"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
     <t>ياسر</t>
   </si>
   <si>
-    <t>تجربة ناجحة</t>
+    <t>مرحباً نجح التحديث</t>
   </si>
 </sst>
 </file>
@@ -87,9 +87,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
@@ -424,12 +427,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C2837BD-C24C-40E9-A47C-56190C4D39DE}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultColWidth="10.3125" defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.3125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.4375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.9375" customWidth="1"/>
+    <col min="4" max="4" width="17.5625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -450,9 +454,69 @@
       <c r="B2" s="1">
         <v>966505887741</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C22" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>